<commit_message>
added metadata (018). Still needs to finish DAS issue before joining back in joined qmd and moving on.
</commit_message>
<xml_diff>
--- a/data/verification/datastet_and_added_summarised/datastet_and_added_filled_raw/charite_dois_ids_distinct_v9.xlsx
+++ b/data/verification/datastet_and_added_summarised/datastet_and_added_filled_raw/charite_dois_ids_distinct_v9.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29318"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\AVIHAY\git\DCC-v3\data\verification\datastet_and_added_summarised\datastet_and_added_filled_raw\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://charitede.sharepoint.com/sites/TeamOpenDataundForschungsdatenmanagement/Shared Documents/DCC analysis/datastet and added identifiers/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3322BA5-DB1C-451A-957B-0E41A0843540}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2695" documentId="11_57DF80A4F9203448D8892CCCE483C471B2B16C48" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D336E1B8-7CFE-4B50-A261-1C7CA944C819}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="30960" windowHeight="16800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,10 +28,10 @@
         <xcalcf:feature name="microsoft.com:RD"/>
         <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6824" uniqueCount="1408">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6869" uniqueCount="1421">
   <si>
     <t>doi_datastet_and_added</t>
   </si>
@@ -4263,6 +4263,45 @@
   </si>
   <si>
     <t>code cannot be found in the publication</t>
+  </si>
+  <si>
+    <t>10.17863/cam.23511</t>
+  </si>
+  <si>
+    <t>University of Cambridge Repository</t>
+  </si>
+  <si>
+    <t>CC BY</t>
+  </si>
+  <si>
+    <t>10.1242/dev.201228</t>
+  </si>
+  <si>
+    <t>10.17863/cam.87955</t>
+  </si>
+  <si>
+    <t>not in DAS</t>
+  </si>
+  <si>
+    <t>10.1038/s41467-020-16929-8</t>
+  </si>
+  <si>
+    <t>10.5281/zenodo.2529950</t>
+  </si>
+  <si>
+    <t>Zenodo</t>
+  </si>
+  <si>
+    <t>10.1016/j.cortex.2021.08.002</t>
+  </si>
+  <si>
+    <t>10.6084/m9.figshare.915436</t>
+  </si>
+  <si>
+    <t>figshare</t>
+  </si>
+  <si>
+    <t>10.1016/j.nicl.2020.102536</t>
   </si>
 </sst>
 </file>
@@ -4348,9 +4387,16 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="4">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -4386,9 +4432,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -4426,9 +4472,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -4461,26 +4507,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -4513,26 +4542,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -4706,7 +4718,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:P968"/>
+  <dimension ref="A1:P967"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40.28515625" bestFit="1" customWidth="1"/>
@@ -32848,30 +32860,192 @@
         <v>0</v>
       </c>
     </row>
+    <row r="963" spans="1:15">
+      <c r="A963" t="s">
+        <v>68</v>
+      </c>
+      <c r="B963" t="s">
+        <v>1408</v>
+      </c>
+      <c r="C963" t="s">
+        <v>17</v>
+      </c>
+      <c r="D963" t="s">
+        <v>35</v>
+      </c>
+      <c r="E963" s="1">
+        <v>45924</v>
+      </c>
+      <c r="F963" t="s">
+        <v>20</v>
+      </c>
+      <c r="G963" t="s">
+        <v>20</v>
+      </c>
+      <c r="H963" t="s">
+        <v>1409</v>
+      </c>
+      <c r="I963" t="s">
+        <v>20</v>
+      </c>
+      <c r="J963" t="s">
+        <v>20</v>
+      </c>
+      <c r="K963" t="s">
+        <v>31</v>
+      </c>
+      <c r="L963" t="s">
+        <v>1410</v>
+      </c>
+      <c r="M963" t="s">
+        <v>20</v>
+      </c>
+      <c r="N963">
+        <v>2023</v>
+      </c>
+    </row>
+    <row r="964" spans="1:15">
+      <c r="A964" t="s">
+        <v>1411</v>
+      </c>
+      <c r="B964" s="7" t="s">
+        <v>1412</v>
+      </c>
+      <c r="C964" t="s">
+        <v>17</v>
+      </c>
+      <c r="D964" t="s">
+        <v>35</v>
+      </c>
+      <c r="E964" s="1">
+        <v>45924</v>
+      </c>
+      <c r="F964" t="s">
+        <v>20</v>
+      </c>
+      <c r="G964" t="s">
+        <v>20</v>
+      </c>
+      <c r="H964" t="s">
+        <v>1409</v>
+      </c>
+      <c r="I964" t="s">
+        <v>1413</v>
+      </c>
+      <c r="J964" t="s">
+        <v>31</v>
+      </c>
+      <c r="K964" t="s">
+        <v>31</v>
+      </c>
+      <c r="L964" t="s">
+        <v>1410</v>
+      </c>
+      <c r="M964" t="s">
+        <v>20</v>
+      </c>
+      <c r="N964">
+        <v>2023</v>
+      </c>
+    </row>
     <row r="965" spans="1:15">
-      <c r="B965" s="7"/>
+      <c r="A965" t="s">
+        <v>1414</v>
+      </c>
+      <c r="B965" t="s">
+        <v>1415</v>
+      </c>
+      <c r="C965" t="s">
+        <v>17</v>
+      </c>
+      <c r="D965" t="s">
+        <v>35</v>
+      </c>
+      <c r="E965" s="1">
+        <v>45924</v>
+      </c>
+      <c r="F965" t="s">
+        <v>19</v>
+      </c>
+      <c r="G965" t="s">
+        <v>100</v>
+      </c>
+      <c r="H965" t="s">
+        <v>1416</v>
+      </c>
+    </row>
+    <row r="966" spans="1:15">
+      <c r="A966" t="s">
+        <v>1417</v>
+      </c>
+      <c r="B966" s="7" t="s">
+        <v>1418</v>
+      </c>
+      <c r="C966" t="s">
+        <v>17</v>
+      </c>
+      <c r="D966" t="s">
+        <v>35</v>
+      </c>
+      <c r="E966" s="1">
+        <v>45924</v>
+      </c>
+      <c r="F966" t="s">
+        <v>19</v>
+      </c>
+      <c r="G966" t="s">
+        <v>100</v>
+      </c>
+      <c r="H966" t="s">
+        <v>1419</v>
+      </c>
     </row>
     <row r="967" spans="1:15">
-      <c r="B967" s="7"/>
-    </row>
-    <row r="968" spans="1:15">
-      <c r="B968" s="7"/>
+      <c r="A967" t="s">
+        <v>1420</v>
+      </c>
+      <c r="B967" t="s">
+        <v>1418</v>
+      </c>
+      <c r="C967" t="s">
+        <v>17</v>
+      </c>
+      <c r="D967" t="s">
+        <v>35</v>
+      </c>
+      <c r="E967" s="1">
+        <v>45924</v>
+      </c>
+      <c r="F967" t="s">
+        <v>19</v>
+      </c>
+      <c r="G967" t="s">
+        <v>100</v>
+      </c>
+      <c r="H967" t="s">
+        <v>1419</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:P962" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <conditionalFormatting sqref="B30:O30 A48:O50 B51:O51 B66:O66 B163:O163 A213:H213 I213:O214 A215:O230 B231:O231 B214:G214 A232:O245 B246:O246 A145:H145 A1:O29 A31:O46 B47:O47 J145:O145 A52:O65 A67:O144 A146:O162 A164:O212 O570:O594 A595:O962 A247:O569 A570:M594">
-    <cfRule type="expression" dxfId="2" priority="1">
+    <cfRule type="expression" dxfId="3" priority="2">
       <formula>$O1=TRUE</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H214">
-    <cfRule type="expression" dxfId="1" priority="3">
+    <cfRule type="expression" dxfId="2" priority="4">
       <formula>$O213=TRUE</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N582:N594">
-    <cfRule type="expression" dxfId="0" priority="5">
+    <cfRule type="expression" dxfId="1" priority="6">
       <formula>$O570=TRUE</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E963:E967">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>$O963=TRUE</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -32879,9 +33053,10 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100029FD0B41DD07841BED16965712E158C" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e0f1011f30fef6dde8223745cec2fc96">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="aaacefca-f467-416c-abd0-2b181dff1e20" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4d5cb4cdee1db726a521ed27371901b5" ns2:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100029FD0B41DD07841BED16965712E158C" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="ae6d51e96c8c66a8de8dfe8311f95192">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="aaacefca-f467-416c-abd0-2b181dff1e20" xmlns:ns3="a0e84d40-090a-490d-8a02-2942ffba970a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1f9e171e4f7fb14517da8847a2c60885" ns2:_="" ns3:_="">
     <xsd:import namespace="aaacefca-f467-416c-abd0-2b181dff1e20"/>
+    <xsd:import namespace="a0e84d40-090a-490d-8a02-2942ffba970a"/>
     <xsd:element name="properties">
       <xsd:complexType>
         <xsd:sequence>
@@ -32892,6 +33067,12 @@
                 <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -32921,6 +33102,50 @@
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="12" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="14" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="2375ea7b-1eef-4e91-915e-32e4cb5a9c34" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="a0e84d40-090a-490d-8a02-2942ffba970a" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="15" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{b1b93042-dae5-4a91-aee7-e8b26f1570c8}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="a0e84d40-090a-490d-8a02-2942ffba970a">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
     </xsd:element>
   </xsd:schema>
   <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
@@ -33023,12 +33248,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -33037,37 +33256,25 @@
 </FormTemplates>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="a0e84d40-090a-490d-8a02-2942ffba970a" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="aaacefca-f467-416c-abd0-2b181dff1e20">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{62DB5D2C-15B8-4357-A22A-D88F7291A956}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="aaacefca-f467-416c-abd0-2b181dff1e20"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F2C5B169-AEF7-4447-855E-125D156E9E64}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{45D27483-4B25-4C13-ADD2-2FFF45E1670E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B07315CF-E1D2-41BC-97DE-837096B66448}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B07315CF-E1D2-41BC-97DE-837096B66448}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{45D27483-4B25-4C13-ADD2-2FFF45E1670E}"/>
 </file>
</xml_diff>